<commit_message>
add video lessons and simple reviews
</commit_message>
<xml_diff>
--- a/hair_shop/wb_exports/change_price.xlsx
+++ b/hair_shop/wb_exports/change_price.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0911271F-FEB2-4DAC-B134-5DC6B837A8E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71609111-E67B-44BF-BAE0-2E867718EAB8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2558,10 +2558,10 @@
     <t>1305х60х2135с</t>
   </si>
   <si>
-    <t>article</t>
-  </si>
-  <si>
-    <t>price</t>
+    <t>артикль</t>
+  </si>
+  <si>
+    <t>цена</t>
   </si>
 </sst>
 </file>

</xml_diff>